<commit_message>
Angles instead of cosines, figure for review response
</commit_message>
<xml_diff>
--- a/ms_tables/table2_disparity_n_small_fam.xlsx
+++ b/ms_tables/table2_disparity_n_small_fam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thomas/Documents/GitHub/GvsP/ms_tables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FF3F68C-323D-8443-88B7-CE2CF7B1DCC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE3A27A0-4E6F-5C4C-9119-F806C0A69081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27320" yWindow="620" windowWidth="27320" windowHeight="19860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38400" yWindow="620" windowWidth="38400" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -649,6 +649,7 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -661,7 +662,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -689,8 +689,8 @@
       <xdr:rowOff>1960</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="707834" cy="181231"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="TextBox 11">
@@ -770,7 +770,7 @@
                               <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>𝑔</m:t>
+                              <m:t>𝑝</m:t>
                             </m:r>
                           </m:sub>
                         </m:sSub>
@@ -828,7 +828,7 @@
                               <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>𝑝</m:t>
+                              <m:t>𝑔</m:t>
                             </m:r>
                           </m:sub>
                         </m:sSub>
@@ -842,7 +842,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="TextBox 11">
@@ -895,37 +895,37 @@
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
+                <a:t>𝑟_𝑝 ) ̂</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>  </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>vs</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
                 <a:t>𝑟_𝑔 ) ̂</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="1" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>  </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>vs</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="1" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t> </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑟_𝑝 ) ̂</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -943,8 +943,8 @@
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="606704" cy="204999"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -993,6 +993,64 @@
                     <m:jc m:val="center"/>
                   </m:oMathParaPr>
                   <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:acc>
+                      <m:accPr>
+                        <m:chr m:val="̂"/>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:accPr>
+                      <m:e>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑟</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑝</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                      </m:e>
+                    </m:acc>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="1" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:sty m:val="p"/>
+                      </m:rPr>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>vs</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="1" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1024,67 +1082,15 @@
                       </a:rPr>
                       <m:t> </m:t>
                     </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:sty m:val="p"/>
-                      </m:rPr>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>vs</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t> </m:t>
-                    </m:r>
-                    <m:acc>
-                      <m:accPr>
-                        <m:chr m:val="̂"/>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:accPr>
-                      <m:e>
-                        <m:sSub>
-                          <m:sSubPr>
-                            <m:ctrlPr>
-                              <a:rPr lang="en-US" sz="1100" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                            </m:ctrlPr>
-                          </m:sSubPr>
-                          <m:e>
-                            <m:r>
-                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                              <m:t>𝑟</m:t>
-                            </m:r>
-                          </m:e>
-                          <m:sub>
-                            <m:r>
-                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                              <m:t>𝑝</m:t>
-                            </m:r>
-                          </m:sub>
-                        </m:sSub>
-                      </m:e>
-                    </m:acc>
                   </m:oMath>
                 </m:oMathPara>
               </a14:m>
-              <a:endParaRPr lang="en-US" sz="1100"/>
+              <a:endParaRPr lang="en-US" sz="1100" i="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="TextBox 12">
@@ -1128,9 +1134,39 @@
             <a:p>
               <a:pPr/>
               <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(</a:t>
+              </a:r>
+              <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
+                <a:t>𝑟_𝑝 ) ̂</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>  </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>vs</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
                 <a:t>𝑟_𝑔</a:t>
               </a:r>
               <a:r>
@@ -1139,25 +1175,7 @@
                 </a:rPr>
                 <a:t>  </a:t>
               </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>vs </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑟_𝑝 ) ̂</a:t>
-              </a:r>
-              <a:endParaRPr lang="en-US" sz="1100"/>
+              <a:endParaRPr lang="en-US" sz="1100" i="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
@@ -1415,20 +1433,20 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>939798</xdr:colOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>1960</xdr:rowOff>
+      <xdr:rowOff>20320</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="707834" cy="181231"/>
+    <xdr:ext cx="219364" cy="175369"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
       <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="15" name="TextBox 14">
+            <xdr:cNvPr id="2" name="TextBox 1">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79398D46-FB59-2D4C-AE79-C13FCB0A0D54}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E296297-6496-BE4D-8B60-6FE9C1F98533}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1436,7 +1454,155 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8072118" y="205160"/>
+              <a:off x="0" y="223520"/>
+              <a:ext cx="219364" cy="175369"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:sSup>
+                      <m:sSupPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:sSupPr>
+                      <m:e>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>h</m:t>
+                        </m:r>
+                      </m:e>
+                      <m:sup>
+                        <m:r>
+                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                          <m:t>2</m:t>
+                        </m:r>
+                      </m:sup>
+                    </m:sSup>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2" name="TextBox 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E296297-6496-BE4D-8B60-6FE9C1F98533}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="0" y="223520"/>
+              <a:ext cx="219364" cy="175369"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:style>
+            <a:lnRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:lnRef>
+            <a:fillRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:fillRef>
+            <a:effectRef idx="0">
+              <a:scrgbClr r="0" g="0" b="0"/>
+            </a:effectRef>
+            <a:fontRef idx="minor">
+              <a:schemeClr val="tx1"/>
+            </a:fontRef>
+          </xdr:style>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>ℎ^2</a:t>
+              </a:r>
+              <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>970278</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>1960</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="707834" cy="181231"/>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="9" name="TextBox 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A84E648-5DEE-A54B-90A2-09F8F9E21F73}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8102598" y="205160"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1502,7 +1668,7 @@
                               <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>𝑔</m:t>
+                              <m:t>𝑝</m:t>
                             </m:r>
                           </m:sub>
                         </m:sSub>
@@ -1560,7 +1726,7 @@
                               <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>𝑝</m:t>
+                              <m:t>𝑔</m:t>
                             </m:r>
                           </m:sub>
                         </m:sSub>
@@ -1574,13 +1740,13 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="15" name="TextBox 14">
+            <xdr:cNvPr id="9" name="TextBox 8">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79398D46-FB59-2D4C-AE79-C13FCB0A0D54}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A84E648-5DEE-A54B-90A2-09F8F9E21F73}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1588,7 +1754,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8072118" y="205160"/>
+              <a:off x="8102598" y="205160"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1627,37 +1793,37 @@
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
+                <a:t>𝑟_𝑝 ) ̂</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>  </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>vs</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
                 <a:t>𝑟_𝑔 ) ̂</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="1" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>  </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>vs</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="1" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t> </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑟_𝑝 ) ̂</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -1670,19 +1836,19 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1361440</xdr:colOff>
+      <xdr:colOff>1391920</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="606704" cy="204999"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="16" name="TextBox 15">
+            <xdr:cNvPr id="10" name="TextBox 9">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC17798D-E208-534D-BE35-6FAA8072FD22}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75191DC3-6531-8C48-9352-50D704D0BC44}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1690,7 +1856,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5984240" y="203200"/>
+              <a:off x="6014720" y="203200"/>
               <a:ext cx="606704" cy="204999"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1725,6 +1891,64 @@
                     <m:jc m:val="center"/>
                   </m:oMathParaPr>
                   <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:acc>
+                      <m:accPr>
+                        <m:chr m:val="̂"/>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:accPr>
+                      <m:e>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑟</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑝</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                      </m:e>
+                    </m:acc>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="1" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:sty m:val="p"/>
+                      </m:rPr>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>vs</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="1" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -1756,73 +1980,21 @@
                       </a:rPr>
                       <m:t> </m:t>
                     </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:sty m:val="p"/>
-                      </m:rPr>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>vs</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t> </m:t>
-                    </m:r>
-                    <m:acc>
-                      <m:accPr>
-                        <m:chr m:val="̂"/>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:accPr>
-                      <m:e>
-                        <m:sSub>
-                          <m:sSubPr>
-                            <m:ctrlPr>
-                              <a:rPr lang="en-US" sz="1100" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                            </m:ctrlPr>
-                          </m:sSubPr>
-                          <m:e>
-                            <m:r>
-                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                              <m:t>𝑟</m:t>
-                            </m:r>
-                          </m:e>
-                          <m:sub>
-                            <m:r>
-                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                              <m:t>𝑝</m:t>
-                            </m:r>
-                          </m:sub>
-                        </m:sSub>
-                      </m:e>
-                    </m:acc>
                   </m:oMath>
                 </m:oMathPara>
               </a14:m>
-              <a:endParaRPr lang="en-US" sz="1100"/>
+              <a:endParaRPr lang="en-US" sz="1100" i="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="16" name="TextBox 15">
+            <xdr:cNvPr id="10" name="TextBox 9">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC17798D-E208-534D-BE35-6FAA8072FD22}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75191DC3-6531-8C48-9352-50D704D0BC44}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1830,7 +2002,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="5984240" y="203200"/>
+              <a:off x="6014720" y="203200"/>
               <a:ext cx="606704" cy="204999"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1860,9 +2032,39 @@
             <a:p>
               <a:pPr/>
               <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(</a:t>
+              </a:r>
+              <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
+                <a:t>𝑟_𝑝 ) ̂</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>  </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>vs</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
                 <a:t>𝑟_𝑔</a:t>
               </a:r>
               <a:r>
@@ -1871,25 +2073,7 @@
                 </a:rPr>
                 <a:t>  </a:t>
               </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>vs </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑟_𝑝 ) ̂</a:t>
-              </a:r>
-              <a:endParaRPr lang="en-US" sz="1100"/>
+              <a:endParaRPr lang="en-US" sz="1100" i="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
@@ -1900,19 +2084,19 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>972768</xdr:colOff>
+      <xdr:colOff>1003248</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>2583</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="707834" cy="181231"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="TextBox 16">
+            <xdr:cNvPr id="11" name="TextBox 10">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D53DE2E-4B07-E248-BD4B-916AA02E1089}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C51B235B-52B9-854F-864C-EBECFEE3B2CD}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -1920,7 +2104,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="7028128" y="205783"/>
+              <a:off x="7058608" y="205783"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2052,13 +2236,13 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="TextBox 16">
+            <xdr:cNvPr id="11" name="TextBox 10">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D53DE2E-4B07-E248-BD4B-916AA02E1089}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C51B235B-52B9-854F-864C-EBECFEE3B2CD}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2066,7 +2250,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="7028128" y="205783"/>
+              <a:off x="7058608" y="205783"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2148,19 +2332,19 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>939798</xdr:colOff>
+      <xdr:colOff>970278</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>1960</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="707834" cy="181231"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="18" name="TextBox 17">
+            <xdr:cNvPr id="21" name="TextBox 20">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BDFE026-9375-CD48-821B-BD42594FDEC8}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{737BE247-E95D-7E40-A7B6-CE6982D84DAF}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2168,7 +2352,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="11628118" y="205160"/>
+              <a:off x="11658598" y="205160"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2234,7 +2418,7 @@
                               <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>𝑔</m:t>
+                              <m:t>𝑝</m:t>
                             </m:r>
                           </m:sub>
                         </m:sSub>
@@ -2292,7 +2476,7 @@
                               <a:rPr lang="en-US" sz="1100" b="0" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>𝑝</m:t>
+                              <m:t>𝑔</m:t>
                             </m:r>
                           </m:sub>
                         </m:sSub>
@@ -2306,13 +2490,13 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="18" name="TextBox 17">
+            <xdr:cNvPr id="21" name="TextBox 20">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BDFE026-9375-CD48-821B-BD42594FDEC8}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{737BE247-E95D-7E40-A7B6-CE6982D84DAF}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2320,7 +2504,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="11628118" y="205160"/>
+              <a:off x="11658598" y="205160"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2359,37 +2543,37 @@
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
+                <a:t>𝑟_𝑝 ) ̂</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>  </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>vs</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
                 <a:t>𝑟_𝑔 ) ̂</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="1" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>  </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>vs</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="1" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t> </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑟_𝑝 ) ̂</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -2402,19 +2586,19 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>1341120</xdr:colOff>
+      <xdr:colOff>1371600</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="606704" cy="204999"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="19" name="TextBox 18">
+            <xdr:cNvPr id="22" name="TextBox 21">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3D4E357-FC4A-F94B-A0DE-B8AEFF596BA9}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0008A1EE-1709-BE4C-8859-C398D6CA886C}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2422,7 +2606,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="9540240" y="203200"/>
+              <a:off x="9570720" y="203200"/>
               <a:ext cx="606704" cy="204999"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2457,6 +2641,64 @@
                     <m:jc m:val="center"/>
                   </m:oMathParaPr>
                   <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:acc>
+                      <m:accPr>
+                        <m:chr m:val="̂"/>
+                        <m:ctrlPr>
+                          <a:rPr lang="en-US" sz="1100" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:accPr>
+                      <m:e>
+                        <m:sSub>
+                          <m:sSubPr>
+                            <m:ctrlPr>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                            </m:ctrlPr>
+                          </m:sSubPr>
+                          <m:e>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑟</m:t>
+                            </m:r>
+                          </m:e>
+                          <m:sub>
+                            <m:r>
+                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>𝑝</m:t>
+                            </m:r>
+                          </m:sub>
+                        </m:sSub>
+                      </m:e>
+                    </m:acc>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="1" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:sty m:val="p"/>
+                      </m:rPr>
+                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>vs</m:t>
+                    </m:r>
+                    <m:r>
+                      <a:rPr lang="en-US" sz="1100" b="1" i="1">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
                     <m:sSub>
                       <m:sSubPr>
                         <m:ctrlPr>
@@ -2488,73 +2730,21 @@
                       </a:rPr>
                       <m:t> </m:t>
                     </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:sty m:val="p"/>
-                      </m:rPr>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t>vs</m:t>
-                    </m:r>
-                    <m:r>
-                      <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t> </m:t>
-                    </m:r>
-                    <m:acc>
-                      <m:accPr>
-                        <m:chr m:val="̂"/>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:accPr>
-                      <m:e>
-                        <m:sSub>
-                          <m:sSubPr>
-                            <m:ctrlPr>
-                              <a:rPr lang="en-US" sz="1100" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                            </m:ctrlPr>
-                          </m:sSubPr>
-                          <m:e>
-                            <m:r>
-                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                              <m:t>𝑟</m:t>
-                            </m:r>
-                          </m:e>
-                          <m:sub>
-                            <m:r>
-                              <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                              </a:rPr>
-                              <m:t>𝑝</m:t>
-                            </m:r>
-                          </m:sub>
-                        </m:sSub>
-                      </m:e>
-                    </m:acc>
                   </m:oMath>
                 </m:oMathPara>
               </a14:m>
-              <a:endParaRPr lang="en-US" sz="1100"/>
+              <a:endParaRPr lang="en-US" sz="1100" i="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="19" name="TextBox 18">
+            <xdr:cNvPr id="22" name="TextBox 21">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C3D4E357-FC4A-F94B-A0DE-B8AEFF596BA9}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0008A1EE-1709-BE4C-8859-C398D6CA886C}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2562,7 +2752,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="9540240" y="203200"/>
+              <a:off x="9570720" y="203200"/>
               <a:ext cx="606704" cy="204999"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2592,9 +2782,39 @@
             <a:p>
               <a:pPr/>
               <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>(</a:t>
+              </a:r>
+              <a:r>
                 <a:rPr lang="en-US" sz="1100" b="0" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
+                <a:t>𝑟_𝑝 ) ̂</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>  </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>vs</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="1" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
                 <a:t>𝑟_𝑔</a:t>
               </a:r>
               <a:r>
@@ -2603,25 +2823,7 @@
                 </a:rPr>
                 <a:t>  </a:t>
               </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>vs </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>(</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>𝑟_𝑝 ) ̂</a:t>
-              </a:r>
-              <a:endParaRPr lang="en-US" sz="1100"/>
+              <a:endParaRPr lang="en-US" sz="1100" i="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
@@ -2632,19 +2834,19 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>972768</xdr:colOff>
+      <xdr:colOff>1003248</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>2583</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="707834" cy="181231"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="20" name="TextBox 19">
+            <xdr:cNvPr id="23" name="TextBox 22">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DA101E6-5E0C-314E-9B31-6B766876706D}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF4743EC-A771-A141-8913-CE54BEA79A89}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2652,7 +2854,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="10584128" y="205783"/>
+              <a:off x="10614608" y="205783"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2784,13 +2986,13 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
-            <xdr:cNvPr id="20" name="TextBox 19">
+            <xdr:cNvPr id="23" name="TextBox 22">
               <a:extLst>
                 <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DA101E6-5E0C-314E-9B31-6B766876706D}"/>
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EF4743EC-A771-A141-8913-CE54BEA79A89}"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPr>
@@ -2798,7 +3000,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="10584128" y="205783"/>
+              <a:off x="10614608" y="205783"/>
               <a:ext cx="707834" cy="181231"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2870,154 +3072,6 @@
                 <a:t>  </a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100" i="0"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>20320</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="219364" cy="175369"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2" name="TextBox 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E296297-6496-BE4D-8B60-6FE9C1F98533}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="0" y="223520"/>
-              <a:ext cx="219364" cy="175369"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr/>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:sSup>
-                      <m:sSupPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:sSupPr>
-                      <m:e>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>h</m:t>
-                        </m:r>
-                      </m:e>
-                      <m:sup>
-                        <m:r>
-                          <a:rPr lang="en-US" sz="1100" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                          <m:t>2</m:t>
-                        </m:r>
-                      </m:sup>
-                    </m:sSup>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="en-US" sz="1100" b="0"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="2" name="TextBox 1">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2E296297-6496-BE4D-8B60-6FE9C1F98533}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="0" y="223520"/>
-              <a:ext cx="219364" cy="175369"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:fillRef>
-            <a:effectRef idx="0">
-              <a:scrgbClr r="0" g="0" b="0"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0" anchor="t">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr/>
-              <a:r>
-                <a:rPr lang="en-US" sz="1100" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t>ℎ^2</a:t>
-              </a:r>
-              <a:endParaRPr lang="en-US" sz="1100" b="0"/>
             </a:p>
           </xdr:txBody>
         </xdr:sp>
@@ -3342,21 +3396,21 @@
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-      <c r="D1" s="15" t="s">
+      <c r="D1" s="16" t="s">
         <v>164</v>
       </c>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="15" t="s">
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="16" t="s">
         <v>165</v>
       </c>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="15" t="s">
+      <c r="H1" s="17"/>
+      <c r="I1" s="17"/>
+      <c r="J1" s="16" t="s">
         <v>166</v>
       </c>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
+      <c r="K1" s="17"/>
+      <c r="L1" s="17"/>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
@@ -3377,10 +3431,10 @@
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A3" s="17">
+      <c r="A3" s="18">
         <v>0.1</v>
       </c>
-      <c r="B3" s="17">
+      <c r="B3" s="18">
         <v>4</v>
       </c>
       <c r="C3" s="3">
@@ -3415,8 +3469,8 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A4" s="13"/>
-      <c r="B4" s="13"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="5">
         <v>60</v>
       </c>
@@ -3449,8 +3503,8 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A5" s="13"/>
-      <c r="B5" s="14"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="15"/>
       <c r="C5" s="7">
         <v>200</v>
       </c>
@@ -3483,8 +3537,8 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A6" s="13"/>
-      <c r="B6" s="17">
+      <c r="A6" s="14"/>
+      <c r="B6" s="18">
         <v>8</v>
       </c>
       <c r="C6" s="3">
@@ -3519,8 +3573,8 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
       <c r="C7" s="5">
         <v>60</v>
       </c>
@@ -3553,8 +3607,8 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="15"/>
       <c r="C8" s="7">
         <v>200</v>
       </c>
@@ -3587,8 +3641,8 @@
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A9" s="13"/>
-      <c r="B9" s="12">
+      <c r="A9" s="14"/>
+      <c r="B9" s="13">
         <v>12</v>
       </c>
       <c r="C9" s="3">
@@ -3623,8 +3677,8 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
+      <c r="A10" s="14"/>
+      <c r="B10" s="14"/>
       <c r="C10" s="5">
         <v>60</v>
       </c>
@@ -3657,8 +3711,8 @@
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A11" s="14"/>
-      <c r="B11" s="14"/>
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
       <c r="C11" s="7">
         <v>200</v>
       </c>
@@ -3691,10 +3745,10 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A12" s="12">
+      <c r="A12" s="13">
         <v>0.5</v>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="18">
         <v>4</v>
       </c>
       <c r="C12" s="3">
@@ -3729,8 +3783,8 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
+      <c r="A13" s="14"/>
+      <c r="B13" s="14"/>
       <c r="C13" s="5">
         <v>60</v>
       </c>
@@ -3763,8 +3817,8 @@
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
+      <c r="A14" s="14"/>
+      <c r="B14" s="15"/>
       <c r="C14" s="7">
         <v>200</v>
       </c>
@@ -3797,8 +3851,8 @@
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A15" s="13"/>
-      <c r="B15" s="17">
+      <c r="A15" s="14"/>
+      <c r="B15" s="18">
         <v>8</v>
       </c>
       <c r="C15" s="3">
@@ -3833,8 +3887,8 @@
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="14"/>
       <c r="C16" s="5">
         <v>60</v>
       </c>
@@ -3867,8 +3921,8 @@
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="15"/>
       <c r="C17" s="7">
         <v>200</v>
       </c>
@@ -3901,8 +3955,8 @@
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="13"/>
-      <c r="B18" s="12">
+      <c r="A18" s="14"/>
+      <c r="B18" s="13">
         <v>12</v>
       </c>
       <c r="C18" s="3">
@@ -3937,8 +3991,8 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="13"/>
-      <c r="B19" s="13"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
       <c r="C19" s="5">
         <v>60</v>
       </c>
@@ -3971,8 +4025,8 @@
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
       <c r="C20" s="7">
         <v>200</v>
       </c>
@@ -4005,7 +4059,7 @@
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="E21" s="18"/>
+      <c r="E21" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="11">

</xml_diff>